<commit_message>
made kr2 suggested changes, ready for more ;)
</commit_message>
<xml_diff>
--- a/t/TestData/sampleValidation/test-meta.xlsx
+++ b/t/TestData/sampleValidation/test-meta.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Tissue_ID</t>
   </si>
@@ -63,6 +63,15 @@
   </si>
   <si>
     <t>test_sample.1.bam</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>test_sample.2.bam</t>
   </si>
 </sst>
 </file>
@@ -383,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -433,6 +442,23 @@
         <v>11</v>
       </c>
     </row>
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>